<commit_message>
Refactor temperature and state retrieval in AirCompressorControl.py
Updated the callback method to use dictionary comprehensions for retrieving temperature and state values, improving code readability and efficiency. This change simplifies the data structure used for returning values to the server.
</commit_message>
<xml_diff>
--- a/Confiles/协议/读地址.xlsx
+++ b/Confiles/协议/读地址.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\空压机\Confiles\协议\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\code\真空罐压缩机\Confiles\协议\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225C426D-CAA0-4CE9-85D4-8873B3BCEF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6E6D76-3FAD-49D7-9E59-845434544276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -128,16 +128,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -145,26 +145,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -473,145 +474,155 @@
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.54296875" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.81640625" style="5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.7265625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.7265625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="55.54296875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="6">
         <v>15</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="6">
         <v>540</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="6">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="6">
         <v>4</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="6">
         <v>6</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="6">
         <v>2</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="6">
         <v>15</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="6">
         <v>142</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="6">
         <v>4</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
     </row>
     <row r="5" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="6">
         <v>15</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="6">
         <v>250</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="6">
         <v>4</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="6">
         <v>18</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="6">
         <v>562</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="6">
         <v>4</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="6">
         <v>15</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="6">
         <v>502</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="6">
         <v>4</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="3" t="s">
         <v>13</v>
       </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Refactor boolean data retrieval in S7_1200.py
Updated the logic for reading boolean data types to prioritize bit indexing from a dedicated column, falling back to parsing the address if necessary. This change enhances the accuracy of data retrieval from the PLC by correctly handling bit indices and byte addresses.
</commit_message>
<xml_diff>
--- a/Confiles/协议/读地址.xlsx
+++ b/Confiles/协议/读地址.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\code\真空罐压缩机\Confiles\协议\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD6E6D76-3FAD-49D7-9E59-845434544276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DBBEEF1-0211-4747-A59D-BE8A2C84C506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
   <si>
     <t>数据名称</t>
   </si>
@@ -46,9 +46,6 @@
     <t>bool</t>
   </si>
   <si>
-    <t>True:上电;False:断电;</t>
-  </si>
-  <si>
     <t>温控状态</t>
   </si>
   <si>
@@ -58,15 +55,9 @@
     <t>0:温控停止;1:温控运行;2:温控故障;</t>
   </si>
   <si>
-    <t>热沉当前设定温度</t>
-  </si>
-  <si>
     <t>real</t>
   </si>
   <si>
-    <t>热沉控温点温度</t>
-  </si>
-  <si>
     <t>冷板当前设定温度</t>
   </si>
   <si>
@@ -74,6 +65,182 @@
   </si>
   <si>
     <t>一体机上电标志</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>控温点当前设定温度</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>控温点温度</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>温控模式</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>bool</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>int</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>:定值;2:程序;</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>True:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>上电</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>;False:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="微软雅黑"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>断电</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>True:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>热沉</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>;False:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>产品</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>True:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>均值</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>;False:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>单点</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>;</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>温控点类型</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>温控类型</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -81,7 +248,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,6 +273,20 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
@@ -145,7 +326,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -156,16 +337,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -471,7 +645,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.81640625" style="1" bestFit="1" customWidth="1"/>
@@ -487,13 +661,13 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -507,122 +681,185 @@
       </c>
     </row>
     <row r="2" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="6">
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3">
         <v>15</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>540</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="7"/>
+        <v>21</v>
+      </c>
+      <c r="G2" s="3"/>
     </row>
     <row r="3" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="3">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="6">
-        <v>4</v>
-      </c>
-      <c r="C3" s="6">
-        <v>6</v>
-      </c>
-      <c r="D3" s="6">
+      <c r="F3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="3">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3">
+        <v>470.1</v>
+      </c>
+      <c r="D4" s="3">
         <v>2</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="7"/>
-    </row>
-    <row r="4" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="6">
+      <c r="E4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="3">
         <v>15</v>
       </c>
-      <c r="C4" s="6">
-        <v>142</v>
-      </c>
-      <c r="D4" s="6">
-        <v>4</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-    </row>
-    <row r="5" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="6">
-        <v>15</v>
-      </c>
-      <c r="C5" s="6">
-        <v>250</v>
-      </c>
-      <c r="D5" s="6">
-        <v>4</v>
+      <c r="C5" s="3">
+        <v>462</v>
+      </c>
+      <c r="D5" s="3">
+        <v>2</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+        <v>18</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="3"/>
     </row>
     <row r="6" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3">
         <v>15</v>
       </c>
-      <c r="B6" s="6">
+      <c r="C6" s="3">
+        <v>126</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3">
+        <v>142</v>
+      </c>
+      <c r="D7" s="3">
+        <v>4</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3">
+        <v>15</v>
+      </c>
+      <c r="C8" s="3">
+        <v>250</v>
+      </c>
+      <c r="D8" s="3">
+        <v>4</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="3">
         <v>18</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C9" s="3">
         <v>562</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D9" s="3">
         <v>4</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+    </row>
+    <row r="10" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
-    </row>
-    <row r="7" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="6">
+      <c r="B10" s="3">
         <v>15</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C10" s="3">
         <v>502</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D10" s="3">
         <v>4</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>